<commit_message>
docs: atualizar status das stories no Excel de planejamento.
Marca S1-S2, S3-01 e S4 como Concluido; S3-02/S3-03 Pendente; Sprint 3 Em andamento.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/pipeline_xgboost_sprints.xlsx
+++ b/docs/pipeline_xgboost_sprints.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +58,11 @@
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +119,18 @@
         <fgColor rgb="00444441"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0090EE90"/>
+        <bgColor rgb="0090EE90"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -143,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -218,6 +233,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -585,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -603,7 +627,18 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="8" customHeight="1"/>
+    <row r="2" ht="8" customHeight="1">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Atualizado em</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -635,6 +670,16 @@
           <t>Objetivo</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Repo</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>bike-sharing-forecast-aws</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -650,9 +695,9 @@
       <c r="C4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Planejado</t>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -680,9 +725,9 @@
       <c r="C5" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Planejado</t>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -710,9 +755,9 @@
       <c r="C6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="11" t="inlineStr">
-        <is>
-          <t>Planejado</t>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -740,9 +785,9 @@
       <c r="C7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="14" t="inlineStr">
-        <is>
-          <t>Planejado</t>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
@@ -859,9 +904,9 @@
 ✔ Script idempotente (sem erro em re-execução)</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -897,9 +942,9 @@
 ✔ IAM role com acesso ao S3 e Glue Catalog</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -935,9 +980,9 @@
 ✔ Falha do job gera notificação SNS</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1044,9 +1089,9 @@
 ✔ Teste unitário cobre cenário de coluna ausente</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1082,9 +1127,9 @@
 ✔ Teste com mês sem dados não quebra o pipeline</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1120,9 +1165,9 @@
 ✔ Partição por ref_date visível no S3</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1229,9 +1274,9 @@
 ✔ Métricas salvas em JSON no S3 (metrics/ref_date/metrics.json)</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1267,9 +1312,9 @@
 ✔ Arquivo .pkl legível com joblib.load</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>Pendente</t>
         </is>
       </c>
     </row>
@@ -1305,9 +1350,9 @@
 ✔ Arquivo salvo e legível no S3</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>Pendente</t>
         </is>
       </c>
     </row>
@@ -1414,9 +1459,9 @@
 ✔ Tabela consultável via Athena sem erro</t>
         </is>
       </c>
-      <c r="G4" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G4" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1452,9 +1497,9 @@
 ✔ Query parametrizável por ref_date via Step Functions</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1490,9 +1535,9 @@
 ✔ Dashboard CloudWatch com métricas do pipeline</t>
         </is>
       </c>
-      <c r="G6" s="19" t="inlineStr">
-        <is>
-          <t>To Do</t>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S3-02/S3-03: serializar modelo, inferencia e pipeline mensal completo.
Adiciona model.pkl (joblib), job Glue predict-xgboost, SFN mensal encadeada S2-S4 com override de ref_date, 57 testes passando, docs e Excel finalizados.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/pipeline_xgboost_sprints.xlsx
+++ b/docs/pipeline_xgboost_sprints.xlsx
@@ -635,7 +635,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-06 (projeto finalizado)</t>
         </is>
       </c>
     </row>
@@ -755,9 +755,9 @@
       <c r="C6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>Em andamento</t>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -1312,9 +1312,9 @@
 ✔ Arquivo .pkl legível com joblib.load</t>
         </is>
       </c>
-      <c r="G5" s="27" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>
@@ -1350,9 +1350,9 @@
 ✔ Arquivo salvo e legível no S3</t>
         </is>
       </c>
-      <c r="G6" s="27" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="G6" s="28" t="inlineStr">
+        <is>
+          <t>Concluido</t>
         </is>
       </c>
     </row>

</xml_diff>